<commit_message>
Update Adjust to contents (gotta love doubles)
</commit_message>
<xml_diff>
--- a/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Misc/AdjustToContents.xlsx
+++ b/ClosedXML/ClosedXML/ClosedXML_Tests/Resource/Examples/Misc/AdjustToContents.xlsx
@@ -3569,14 +3569,14 @@
     <x:col min="1" max="1" width="2.9306249999999996" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="16.150624999999998" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="17.315676440444804" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18.195145171689223" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18.195145171689227" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="17.902475307480557" style="0" customWidth="1"/>
     <x:col min="6" max="6" width="17.495860622181581" style="0" customWidth="1"/>
     <x:col min="7" max="7" width="16.978395699068074" style="0" customWidth="1"/>
     <x:col min="8" max="8" width="16.3540187586588" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="15.627481686479374" style="0" customWidth="1"/>
-    <x:col min="10" max="10" width="14.80431386834416" style="0" customWidth="1"/>
-    <x:col min="11" max="11" width="13.890780108391489" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="14.804313868344162" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="13.890780108391487" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="12.893832950141361" style="0" customWidth="1"/>
     <x:col min="13" max="13" width="11.821059763441216" style="0" customWidth="1"/>
     <x:col min="14" max="14" width="10.680625000000003" style="0" customWidth="1"/>
@@ -3665,18 +3665,18 @@
   <x:cols>
     <x:col min="1" max="1" width="2.9306249999999996" style="0" customWidth="1"/>
     <x:col min="2" max="2" width="51.020625" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="61.832985562903978" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="61.832985562903971" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="61.271495301031983" style="0" customWidth="1"/>
-    <x:col min="5" max="5" width="60.340427494313964" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="59.04686813095315" style="0" customWidth="1"/>
-    <x:col min="7" max="7" width="57.400661978777208" style="0" customWidth="1"/>
-    <x:col min="8" max="8" width="55.414337660610677" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="60.340427494313957" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="59.046868130953143" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="57.400661978777215" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="55.41433766061067" style="0" customWidth="1"/>
     <x:col min="9" max="9" width="53.103012303890189" style="0" customWidth="1"/>
-    <x:col min="10" max="10" width="50.484276490196805" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="50.484276490196812" style="0" customWidth="1"/>
     <x:col min="11" max="11" width="47.578060380308663" style="0" customWidth="1"/>
     <x:col min="12" max="12" width="44.406482033643258" style="0" customWidth="1"/>
-    <x:col min="13" max="13" width="40.993679076470087" style="0" customWidth="1"/>
-    <x:col min="14" max="14" width="37.365625000000009" style="0" customWidth="1"/>
+    <x:col min="13" max="13" width="40.99367907647008" style="0" customWidth="1"/>
+    <x:col min="14" max="14" width="37.365625" style="0" customWidth="1"/>
     <x:col min="15" max="15" width="33.549931486433891" style="0" customWidth="1"/>
     <x:col min="16" max="16" width="29.575638267388729" style="0" customWidth="1"/>
     <x:col min="17" max="17" width="25.4729921140053" style="0" customWidth="1"/>

</xml_diff>